<commit_message>
Meuleman et al. (2009)
</commit_message>
<xml_diff>
--- a/slr/ei/data.xlsx
+++ b/slr/ei/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joechan/Documents/development/researchplymouth/slr/ei/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFDC8633-C2E1-044B-A4DD-CC6359D1C171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6693F55-D430-E440-AFCB-7299A301804F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2000" yWindow="1700" windowWidth="45020" windowHeight="28340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4983" uniqueCount="2308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4994" uniqueCount="2319">
   <si>
     <t>#</t>
   </si>
@@ -7010,6 +7010,39 @@
   </si>
   <si>
     <t xml:space="preserve">Emphasising that entrepreneurial discovery is a crucial antecedent to opportunity creation (Alvarez and Barney, 2007), the research highlights the necessity of integrating internal conceptualisation with external data emergence (Gavetti and Levinthal, 2000). Moving beyond the unidimensional, dichotomic frameworks posited in earlier literature (Shaver and Scott, 1991), this study conceptualises a multidimensional four-quadrant model: deliberate search, eureka, legacy, and serendipitous discovery (Alvarez and Barney, 2008). This framework establishes a more holistic perspective within entrepreneurial discovery theory (Murphy, 2011). </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Within the field of familial entrepreneurial dynamics, this research utilises longitudinal data from the U.S. Panel Study of Income Dynamics (“PSID”) to examine the relationship between parental and filial entrepreneurial behaviours (Mungai and Velamuri, 2011). Drawing on mechanisms about familial pervasive effects (Aldrich and Cliff, 2003) and social role modelling (Bandura, 1986), the authors contend that parental entrepreneurship significantly enhances a child’s entrepreneurial propensity. </t>
+  </si>
+  <si>
+    <t>Research in technological academic entrepreneurship suggests that homogeneity among academic entrepreneurs may hinder social capital development (Mosey and Wright, 2007). In examining the relationship between human capital and social capital, the authors argue that entrepreneurial behaviours build social network; however, they emphasise that professional backgrounds in industry versus entrepreneurship produce notably different human capital profiles.</t>
+  </si>
+  <si>
+    <t>Drawing on affective events theory (Weiss and Cropanzano, 1996), this research develops an entrepreneurial experience model that emphasises the stream of events within pre-venture “lived experience”. It posits that a series of events manifesting as entrepreneurial behaviours positively impacts outcomes and performance (Morris et al., 2012). To examine these propositions, the researchers suggest utilising qualitative methodologies, such as life story approach (Rae and Carswell, 2000) and the critical incidents technique (Cope and Watts, 2000).</t>
+  </si>
+  <si>
+    <t>Within the context of entrepreneurial orientation (“EO”) and firm performance (“FP”), this research conceptualises an EO-FP causal framework incorporating strategy, environmental hostility, dynamism, and resources and capabilities. Utilising a firm-level dataset from Centra targeting small- and medium-sized enterprises (“SMEs”) in Spain between 1998 and 2001 (n=434), the findings demonstrates a positive EO-FP relationship (Covin and Slevin, 1989). Further, the results indicate that environmental factors influence strategy (Baum et al., 2001), thereby supporting the multidimensional conceptualisation of EO (Lumpkin and Dess, 1996).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Within the context of a regional non-profitable medical system in the U.S., this research conceptualises entrepreneurial orientation (“EO”) through three dimensions: risk-taking, innovativeness, and proactiveness (Lumpkin and Dess, 1996). The study examines these as  independent constructs to explore their impact on quitting intention and role ambiguity among both managerial (n=332) and frontline staff (n=1,643) (Monsen and Wayne Boss, 2009). </t>
+  </si>
+  <si>
+    <t>Drawings on entrepreneurial utility-maximisation (Douglas and Shepherd, 2000) within economic theory (Casson, 2003), this research argues that profit-sharing and other incentives serve as primary drivers of work effort (Monsen et al., 2010). Utilising a quantitative experiment involving MBA students  in the U.S. (n=61), this study explores how moderating effects of effort and risk influence the willingness to engage in entrepreneurial behaviours. The empirical findings indicate that a higher expectation of success correlates with a greater willingness to perform entrepreneurial actions.</t>
+  </si>
+  <si>
+    <t>From a cognitive perspective (Neisser, 2014) in entrepreneurial research concerning knowledge structure and decision-making (Mitchell et al., 2002), scholars have recently utilised four distinct approaches to examine entrepreneurial cognition (Mitchell et al., 2007). These include heuristics (Tversky and Kahneman, 1973; Tversky and Kahneman, 1974), entrepreneurial alertness (Kirzner, 1979; Kirzner, 1985), entrepreneurial expertise (Mitchell, 1994; Mitchell et al., 2000), and effectuation (Sarasvathy, 2001; Sarasvathy, 2002). Furthermore, research has expanded to the roles of emotion and affect (Baron, 2008), and the nature of entrepreneurial action (McMullen and Shepherd, 2006).</t>
+  </si>
+  <si>
+    <t>Utilising a dataset from a U.S. medical school covering 1995 to 2004, this research examines how collaboration between academic and industrial scientists influence publication and patents outcomes (Mindruta, 2013). The empirical findings corroborate that scientific publications from both academic and industry produce equivalent value; however, industrial patents interestingly tend to generate higher value than academic publications (Gittelman and Kogut, 2003).</t>
+  </si>
+  <si>
+    <t>Utilising publicly available data for Fortune 1000 companies between 1996 and 2000 (n=898), this research examines the interplay between firm ownership types and entrepreneurial orientation (“EO”), measured by three constructs: innovation, proactiveness, and risk-taking (Rauch et al., 2009b). Posting that role and social identities influence both EO and firm performance, the empirical findings indicate that enterprises owned by a single founder often exhibit higher levels of EO and superior performance (Miller and Le Breton-Miller, 2011).</t>
+  </si>
+  <si>
+    <t>Grounded in the premise that human capital is a primary driver of firm performance (Unger et al., 2011; van der Sluis et al., 2008), the research examines how the education levels of key stakeholders—specifically executives, employees, and consumers—influence entrepreneurial longevity and performance (Millán et al., 2014). Utilising panel data from the European Community Household Panel (“ECHP”) covering the period from 1994 to 2001 (n=13,676), the empirical findings indicate that higher education levels positively impact entrepreneurial outcomes consistent with existing literature (van Praag and van Stel, 2013).</t>
+  </si>
+  <si>
+    <t>In the context of private equity fund acquisitions in the U.K., the research synthesises agency theory (Fox and Marcus, 1992; Jensen, 1993) and strategic entrepreneurship (Ireland et al., 2003), recognising the importance of resources and capabilities and their complementary contributions (Meuleman et al., 2009). Utilising the archival data from private equity fund acquisitions over a decade (1993-2003, n=238) to examine performance implications, the empirical findings indicate that divisional acquisitions often improve efficiency rather than profitability in terms of value creation in entrepreneurship (Castanias and Helfat, 2001).</t>
   </si>
 </sst>
 </file>
@@ -16571,7 +16604,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="160" spans="1:20" ht="102" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:20" ht="170" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>1108</v>
       </c>
@@ -16590,6 +16623,12 @@
       <c r="F160" s="3" t="s">
         <v>2022</v>
       </c>
+      <c r="G160" s="3">
+        <v>4</v>
+      </c>
+      <c r="H160" s="3" t="s">
+        <v>2318</v>
+      </c>
       <c r="I160" s="3" t="s">
         <v>1519</v>
       </c>
@@ -16625,7 +16664,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="161" spans="1:20" ht="153" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:20" ht="170" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>1109</v>
       </c>
@@ -16644,6 +16683,12 @@
       <c r="F161" s="3" t="s">
         <v>2019</v>
       </c>
+      <c r="G161" s="3">
+        <v>4</v>
+      </c>
+      <c r="H161" s="3" t="s">
+        <v>2317</v>
+      </c>
       <c r="I161" s="3" t="s">
         <v>1520</v>
       </c>
@@ -16682,7 +16727,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="162" spans="1:20" ht="119" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:20" ht="153" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>1110</v>
       </c>
@@ -16700,6 +16745,12 @@
       </c>
       <c r="F162" s="3" t="s">
         <v>2024</v>
+      </c>
+      <c r="G162" s="3">
+        <v>3</v>
+      </c>
+      <c r="H162" s="3" t="s">
+        <v>2316</v>
       </c>
       <c r="I162" s="3" t="s">
         <v>1522</v>
@@ -16755,6 +16806,12 @@
       <c r="F163" s="3" t="s">
         <v>2021</v>
       </c>
+      <c r="G163" s="3">
+        <v>3</v>
+      </c>
+      <c r="H163" s="3" t="s">
+        <v>2315</v>
+      </c>
       <c r="I163" s="3" t="s">
         <v>1523</v>
       </c>
@@ -16793,7 +16850,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="164" spans="1:20" ht="170" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:20" ht="187" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>1112</v>
       </c>
@@ -16812,6 +16869,12 @@
       <c r="F164" s="3" t="s">
         <v>2026</v>
       </c>
+      <c r="G164" s="3">
+        <v>5</v>
+      </c>
+      <c r="H164" s="3" t="s">
+        <v>2314</v>
+      </c>
       <c r="I164" s="3" t="s">
         <v>1525</v>
       </c>
@@ -16847,7 +16910,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="165" spans="1:20" ht="102" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:20" ht="153" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>1113</v>
       </c>
@@ -16865,6 +16928,12 @@
       </c>
       <c r="F165" s="3" t="s">
         <v>2013</v>
+      </c>
+      <c r="G165" s="3">
+        <v>4</v>
+      </c>
+      <c r="H165" s="3" t="s">
+        <v>2313</v>
       </c>
       <c r="I165" s="3" t="s">
         <v>1529</v>
@@ -16920,6 +16989,12 @@
       <c r="F166" s="3" t="s">
         <v>2022</v>
       </c>
+      <c r="G166" s="3">
+        <v>2</v>
+      </c>
+      <c r="H166" s="3" t="s">
+        <v>2312</v>
+      </c>
       <c r="I166" s="3" t="s">
         <v>1528</v>
       </c>
@@ -16955,7 +17030,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="167" spans="1:20" ht="119" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:20" ht="170" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>1115</v>
       </c>
@@ -16974,6 +17049,12 @@
       <c r="F167" s="3" t="s">
         <v>2029</v>
       </c>
+      <c r="G167" s="3">
+        <v>4</v>
+      </c>
+      <c r="H167" s="3" t="s">
+        <v>2311</v>
+      </c>
       <c r="I167" s="3" t="s">
         <v>1530</v>
       </c>
@@ -17009,7 +17090,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="168" spans="1:20" ht="119" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:20" ht="153" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>1116</v>
       </c>
@@ -17027,6 +17108,12 @@
       </c>
       <c r="F168" s="3" t="s">
         <v>2020</v>
+      </c>
+      <c r="G168" s="3">
+        <v>3</v>
+      </c>
+      <c r="H168" s="3" t="s">
+        <v>2310</v>
       </c>
       <c r="I168" s="3" t="s">
         <v>1531</v>
@@ -17082,6 +17169,12 @@
       <c r="F169" s="3" t="s">
         <v>2026</v>
       </c>
+      <c r="G169" s="3">
+        <v>3</v>
+      </c>
+      <c r="H169" s="3" t="s">
+        <v>2309</v>
+      </c>
       <c r="I169" s="3" t="s">
         <v>1532</v>
       </c>
@@ -17135,6 +17228,12 @@
       </c>
       <c r="F170" s="3" t="s">
         <v>2024</v>
+      </c>
+      <c r="G170" s="3">
+        <v>5</v>
+      </c>
+      <c r="H170" s="3" t="s">
+        <v>2308</v>
       </c>
       <c r="I170" s="3" t="s">
         <v>1533</v>

</xml_diff>